<commit_message>
Treat INFLAM_ENV and control classes as deliberate no-calls
Mark INFLAM_ENV as NA in the crosswalk like the control tissues, distinguish
deliberate no-calls from unassigned classes, and ignore NIH control codes so
a mis-keyed crosswalk row cannot subtype them.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analyses/molecular-subtyping-methylation/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
+++ b/analyses/molecular-subtyping-methylation/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
@@ -7265,7 +7265,9 @@
       <c r="E99" s="1" t="s">
         <v>613</v>
       </c>
-      <c r="F99" s="1"/>
+      <c r="F99" s="1" t="s">
+        <v>201</v>
+      </c>
       <c r="G99" s="1"/>
       <c r="H99" s="1" t="s">
         <v>614</v>

</xml_diff>

<commit_message>
Mark control and inflammatory microenvironment classes as Control
These indicate low tumor purity, so flag them as controls (methyl_control)
instead of generic no-calls.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analyses/molecular-subtyping-methylation/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
+++ b/analyses/molecular-subtyping-methylation/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="1083">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="1084">
   <si>
     <t xml:space="preserve">Abbreviation_internal_NIHv3</t>
   </si>
@@ -3261,6 +3261,9 @@
   </si>
   <si>
     <t xml:space="preserve">The "mc sinonasal undifferentiated carcinoma, IDH-mutant" emerges as one distinct group among the sinonasal undifferentiated carcinomas. This group includes tumors diagnosed as sinonasal undifferentiated carcinoma, olfactory neuroblastomas, neuroendocrine carcinomas or adenocarcinomas. The tumors carry an IDH2R172 mutation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control</t>
   </si>
 </sst>
 </file>
@@ -4669,7 +4672,7 @@
         <v>200</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>201</v>
+        <v>1083</v>
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1" t="s">
@@ -4704,7 +4707,7 @@
         <v>207</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>201</v>
+        <v>1083</v>
       </c>
       <c r="G29" s="1"/>
       <c r="H29" s="1" t="s">
@@ -4741,7 +4744,7 @@
         <v>213</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>201</v>
+        <v>1083</v>
       </c>
       <c r="G30" s="1"/>
       <c r="H30" s="1" t="s">
@@ -4778,7 +4781,7 @@
         <v>219</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>201</v>
+        <v>1083</v>
       </c>
       <c r="G31" s="1"/>
       <c r="H31" s="1" t="s">
@@ -4815,7 +4818,7 @@
         <v>225</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>201</v>
+        <v>1083</v>
       </c>
       <c r="G32" s="1"/>
       <c r="H32" s="1" t="s">
@@ -4850,7 +4853,7 @@
         <v>231</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>201</v>
+        <v>1083</v>
       </c>
       <c r="G33" s="1"/>
       <c r="H33" s="1" t="s">
@@ -4885,7 +4888,7 @@
         <v>237</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>201</v>
+        <v>1083</v>
       </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1" t="s">
@@ -4920,7 +4923,7 @@
         <v>243</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>201</v>
+        <v>1083</v>
       </c>
       <c r="G35" s="1"/>
       <c r="H35" s="1" t="s">
@@ -4955,7 +4958,7 @@
         <v>251</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>201</v>
+        <v>1083</v>
       </c>
       <c r="G36" s="1"/>
       <c r="H36" s="1" t="s">
@@ -4992,7 +4995,7 @@
         <v>257</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>201</v>
+        <v>1083</v>
       </c>
       <c r="G37" s="1"/>
       <c r="H37" s="1" t="s">
@@ -7266,7 +7269,7 @@
         <v>613</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>201</v>
+        <v>1083</v>
       </c>
       <c r="G99" s="1"/>
       <c r="H99" s="1" t="s">

</xml_diff>